<commit_message>
Druck direkt aus Vorlage, 4 Druckknöpfe, Barcode-Fix
- Drucke direkt aus Etikette_Vorlage.xlsx via Excel COM (keine temp. Datei)
- 4 Buttons: DE/FR jeweils Position oder alle Positionen eines Auftrags
- Jede Position wird in ihrer Menge gedruckt
- Kaputte Barcode-Formeln durch Platzhalter ersetzt

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Etikette_Vorlage.xlsx
+++ b/Etikette_Vorlage.xlsx
@@ -2,19 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28695" yWindow="-16200" windowWidth="29010" windowHeight="15585" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Glas-Etikette" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Glas-Etikette FR" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId3"/>
+  </externalReferences>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Glas-Etikette'!$A$1:$K$23</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Glas-Etikette FR'!$A$1:$K$23</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -27,7 +29,7 @@
     <numFmt numFmtId="167" formatCode="0.0"/>
     <numFmt numFmtId="168" formatCode="0000"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -83,12 +85,6 @@
       <color theme="1"/>
       <sz val="8"/>
     </font>
-    <font>
-      <name val="Code 39-hoch-Logitogo"/>
-      <charset val="2"/>
-      <color theme="1"/>
-      <sz val="26"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -110,80 +106,66 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" textRotation="180"/>
-      <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" textRotation="180"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" textRotation="180"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-      <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" textRotation="180"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" textRotation="180"/>
-      <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" textRotation="180"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-      <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -192,36 +174,12 @@
     <xf numFmtId="168" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" textRotation="180"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" textRotation="180"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -293,6 +251,199 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <to>
+      <col>1</col>
+      <colOff>356230</colOff>
+      <row>4</row>
+      <rowOff>173925</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Grafik 1"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1127755" cy="774000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>6</col>
+      <colOff>114300</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <to>
+      <col>6</col>
+      <colOff>474300</colOff>
+      <row>22</row>
+      <rowOff>133350</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Bild 1" descr="Ce Icon"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill rotWithShape="1">
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:srcRect t="12943" b="12416"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2828925" y="3324225"/>
+          <a:ext cx="360000" cy="276225"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <to>
+      <col>1</col>
+      <colOff>356230</colOff>
+      <row>4</row>
+      <rowOff>173925</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Grafik 1"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1127755" cy="774000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>6</col>
+      <colOff>114300</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <to>
+      <col>6</col>
+      <colOff>474300</colOff>
+      <row>22</row>
+      <rowOff>133350</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Bild 1" descr="Ce Icon"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill rotWithShape="1">
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:srcRect t="12943" b="12416"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2828925" y="3324225"/>
+          <a:ext cx="360000" cy="276225"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <externalBook r:id="rId1">
+    <sheetNames>
+      <sheetName val="ID"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0" refreshError="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -585,276 +736,207 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="11.5703125" customWidth="1" min="1" max="1"/>
-    <col width="7.5703125" customWidth="1" min="2" max="2"/>
-    <col width="1.140625" customWidth="1" min="3" max="3"/>
-    <col width="11.5703125" customWidth="1" min="4" max="4"/>
-    <col width="7.5703125" customWidth="1" min="5" max="5"/>
-    <col width="1.28515625" customWidth="1" min="6" max="6"/>
-    <col width="11.5703125" customWidth="1" min="7" max="7"/>
-    <col width="7.5703125" customWidth="1" min="8" max="8"/>
-    <col width="6.42578125" customWidth="1" min="9" max="9"/>
-    <col width="1.140625" customWidth="1" min="10" max="10"/>
-    <col width="4.42578125" customWidth="1" min="11" max="11"/>
-    <col width="12.7109375" customWidth="1" min="12" max="12"/>
+    <col width="11.5703125" customWidth="1" style="7" min="1" max="1"/>
+    <col width="7.5703125" customWidth="1" style="7" min="2" max="2"/>
+    <col width="1.140625" customWidth="1" style="7" min="3" max="3"/>
+    <col width="11.5703125" customWidth="1" style="7" min="4" max="4"/>
+    <col width="7.5703125" customWidth="1" style="7" min="5" max="5"/>
+    <col width="1.28515625" customWidth="1" style="7" min="6" max="6"/>
+    <col width="11.5703125" customWidth="1" style="7" min="7" max="7"/>
+    <col width="7.5703125" customWidth="1" style="7" min="8" max="8"/>
+    <col width="6.42578125" customWidth="1" style="7" min="9" max="9"/>
+    <col width="1.140625" customWidth="1" style="7" min="10" max="10"/>
+    <col width="4.42578125" customWidth="1" style="7" min="11" max="11"/>
+    <col width="12.7109375" customWidth="1" style="7" min="12" max="12"/>
+    <col width="9.140625" customWidth="1" style="7" min="13" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.1" customHeight="1">
+    <row r="1" ht="14.1" customHeight="1" s="7">
       <c r="A1" s="1" t="n"/>
-      <c r="E1" s="2">
-        <f>ID!M19</f>
-        <v/>
-      </c>
-      <c r="F1" s="3" t="n"/>
-      <c r="G1" s="3" t="n"/>
-      <c r="H1" s="3" t="n"/>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>*000000000000*</t>
+        </is>
+      </c>
       <c r="I1" s="4">
         <f>G4</f>
         <v/>
       </c>
       <c r="J1" s="5" t="n"/>
-      <c r="K1" s="6">
-        <f>ID!M19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="2" ht="14.1" customHeight="1">
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-    </row>
-    <row r="3" ht="5.85" customHeight="1">
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>*000000000000*</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14.1" customHeight="1" s="7"/>
+    <row r="3" ht="5.85" customHeight="1" s="7">
       <c r="E3" s="1" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-    </row>
-    <row r="4" ht="15.6" customHeight="1">
-      <c r="E4" s="7" t="inlineStr">
+    </row>
+    <row r="4" ht="15.6" customHeight="1" s="7">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>AU/Pos</t>
         </is>
       </c>
-      <c r="G4" s="8" t="n">
+      <c r="G4" s="9" t="n">
         <v>143430</v>
       </c>
-      <c r="H4" s="8" t="n">
+      <c r="H4" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="I4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
-    </row>
-    <row r="5" ht="15" customHeight="1">
-      <c r="E5" s="7" t="inlineStr">
+    </row>
+    <row r="5" ht="15" customHeight="1" s="7">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Termin</t>
         </is>
       </c>
-      <c r="G5" s="27" t="n">
+      <c r="G5" s="10" t="n">
         <v>46107</v>
       </c>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="K5" s="3" t="n"/>
-    </row>
-    <row r="6" ht="15" customHeight="1">
+    </row>
+    <row r="6" ht="15" customHeight="1" s="7">
       <c r="A6" s="1" t="n"/>
-      <c r="E6" s="7" t="n"/>
-      <c r="G6" s="10" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="K6" s="3" t="n"/>
-    </row>
-    <row r="7" ht="11.85" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="E6" s="8" t="n"/>
+      <c r="G6" s="11" t="n"/>
+    </row>
+    <row r="7" ht="11.85" customHeight="1" s="7">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Kunde</t>
         </is>
       </c>
-      <c r="I7" s="3" t="n"/>
-      <c r="K7" s="3" t="n"/>
-    </row>
-    <row r="8" ht="15.6" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
+    </row>
+    <row r="8" ht="15.6" customHeight="1" s="7">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>Glas Trösch SA, succursale Bulle</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
-      <c r="I8" s="11" t="n"/>
-      <c r="K8" s="3" t="n"/>
-    </row>
-    <row r="9" ht="5.85" customHeight="1">
-      <c r="A9" s="7" t="n"/>
-      <c r="I9" s="28">
+      <c r="I8" s="12" t="n"/>
+    </row>
+    <row r="9" ht="5.85" customHeight="1" s="7">
+      <c r="A9" s="8" t="n"/>
+      <c r="I9" s="13">
         <f>H4</f>
         <v/>
       </c>
-      <c r="K9" s="3" t="n"/>
-    </row>
-    <row r="10" ht="14.1" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
+    </row>
+    <row r="10" ht="14.1" customHeight="1" s="7">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Kommission</t>
         </is>
       </c>
-      <c r="I10" s="3" t="n"/>
-      <c r="K10" s="3" t="n"/>
-    </row>
-    <row r="11" ht="15.6" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
+    </row>
+    <row r="11" ht="15.6" customHeight="1" s="7">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>635953 / ISO CDR</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
-      <c r="I11" s="3" t="n"/>
-      <c r="K11" s="3" t="n"/>
-    </row>
-    <row r="12" ht="5.85" customHeight="1">
-      <c r="A12" s="7" t="n"/>
-      <c r="I12" s="3" t="n"/>
-      <c r="K12" s="3" t="n"/>
-    </row>
-    <row r="13" ht="14.1" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
+    </row>
+    <row r="12" ht="5.85" customHeight="1" s="7">
+      <c r="A12" s="8" t="n"/>
+    </row>
+    <row r="13" ht="14.1" customHeight="1" s="7">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Kunden-Pos.</t>
         </is>
       </c>
-      <c r="I13" s="3" t="n"/>
-      <c r="K13" s="3" t="n"/>
-    </row>
-    <row r="14" ht="15.6" customHeight="1">
-      <c r="A14" s="10" t="n"/>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
-      <c r="K14" s="3" t="n"/>
-    </row>
-    <row r="15" ht="13.5" customHeight="1">
-      <c r="A15" s="13" t="n"/>
-      <c r="I15" s="3" t="n"/>
-      <c r="K15" s="14" t="n">
-        <v>260127143921</v>
-      </c>
-    </row>
-    <row r="16" ht="14.1" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
+    </row>
+    <row r="14" ht="15.6" customHeight="1" s="7">
+      <c r="A14" s="11" t="n"/>
+    </row>
+    <row r="15" ht="13.5" customHeight="1" s="7">
+      <c r="A15" s="14" t="n"/>
+      <c r="K15" s="15" t="n"/>
+    </row>
+    <row r="16" ht="14.1" customHeight="1" s="7">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Verbund- und Verbundsicherheitsglas mit Anforderung an den Feuerwiderstand</t>
         </is>
       </c>
-      <c r="K16" s="3" t="n"/>
-    </row>
-    <row r="17" ht="15.6" customHeight="1">
-      <c r="A17" s="15" t="inlineStr">
+    </row>
+    <row r="17" ht="15.6" customHeight="1" s="7">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>FSF 30-15  *** ISO 1 ***</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n"/>
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="n"/>
-      <c r="F17" s="3" t="n"/>
-      <c r="G17" s="3" t="n"/>
-      <c r="H17" s="3" t="n"/>
-      <c r="I17" s="3" t="n"/>
-      <c r="K17" s="3" t="n"/>
-    </row>
-    <row r="18" ht="5.85" customHeight="1">
-      <c r="A18" s="7" t="n"/>
-      <c r="K18" s="3" t="n"/>
-    </row>
-    <row r="19" ht="15.6" customHeight="1">
-      <c r="A19" s="16" t="inlineStr">
+    </row>
+    <row r="18" ht="5.85" customHeight="1" s="7">
+      <c r="A18" s="8" t="n"/>
+    </row>
+    <row r="19" ht="15.6" customHeight="1" s="7">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>Menge [Stk]</t>
         </is>
       </c>
-      <c r="B19" s="17" t="n">
+      <c r="B19" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="D19" s="16" t="inlineStr">
+      <c r="D19" s="17" t="inlineStr">
         <is>
           <t>Breite [mm]</t>
         </is>
       </c>
-      <c r="E19" s="18" t="n">
+      <c r="E19" s="19" t="n">
         <v>1728</v>
       </c>
-      <c r="G19" s="16" t="inlineStr">
+      <c r="G19" s="17" t="inlineStr">
         <is>
           <t>Höhe [mm]</t>
         </is>
       </c>
-      <c r="H19" s="18" t="n">
+      <c r="H19" s="19" t="n">
         <v>630</v>
       </c>
-      <c r="K19" s="3" t="n"/>
-    </row>
-    <row r="20" ht="15.6" customHeight="1">
-      <c r="A20" s="16" t="inlineStr">
+    </row>
+    <row r="20" ht="15.6" customHeight="1" s="7">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Fläche [m²]</t>
         </is>
       </c>
-      <c r="B20" s="19">
+      <c r="B20" s="20">
         <f>(E19/1000)*(H19/1000)</f>
         <v/>
       </c>
-      <c r="D20" s="16" t="inlineStr">
+      <c r="D20" s="17" t="inlineStr">
         <is>
           <t>Umfang [lfm]</t>
         </is>
       </c>
-      <c r="E20" s="19">
+      <c r="E20" s="20">
         <f>(E19/1000)*2+(H19/1000)*2</f>
         <v/>
       </c>
-      <c r="G20" s="16" t="inlineStr">
+      <c r="G20" s="17" t="inlineStr">
         <is>
           <t>Gewicht [kg]</t>
         </is>
       </c>
-      <c r="H20" s="29" t="n">
+      <c r="H20" s="21" t="n">
         <v>38.1</v>
       </c>
-      <c r="K20" s="3" t="n"/>
-    </row>
-    <row r="21" ht="13.5" customHeight="1">
+    </row>
+    <row r="21" ht="13.5" customHeight="1" s="7">
       <c r="A21" s="1" t="n"/>
-      <c r="K21" s="3" t="n"/>
-    </row>
-    <row r="22" ht="11.85" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
+    </row>
+    <row r="22" ht="11.85" customHeight="1" s="7">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Nach dem Einbau ist das Etikett sofort zu entfernen.</t>
         </is>
       </c>
-      <c r="G22" s="21" t="n">
+      <c r="G22" s="22" t="n">
         <v>24</v>
       </c>
       <c r="H22" s="1" t="inlineStr">
@@ -862,18 +944,16 @@
           <t>EN 14449</t>
         </is>
       </c>
-      <c r="K22" s="3" t="n"/>
-    </row>
-    <row r="23" ht="11.85" customHeight="1">
-      <c r="A23" s="22" t="inlineStr">
+    </row>
+    <row r="23" ht="11.85" customHeight="1" s="7">
+      <c r="A23" s="23" t="inlineStr">
         <is>
           <t>CDR Glas AG | 3253 Schnottwil | 032 312 03 00 | www.cdr.ch</t>
         </is>
       </c>
-      <c r="G23" s="30" t="n">
+      <c r="G23" s="24" t="n">
         <v>757</v>
       </c>
-      <c r="K23" s="3" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="30">
@@ -901,8 +981,8 @@
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="K1:K14"/>
+    <mergeCell ref="A8:H8"/>
     <mergeCell ref="K15:K23"/>
-    <mergeCell ref="A8:H8"/>
     <mergeCell ref="A1:D5"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A13:H13"/>
@@ -910,6 +990,7 @@
   </mergeCells>
   <pageMargins left="0.07874015748031496" right="0.07874015748031496" top="0.07874015748031496" bottom="0" header="0" footer="0"/>
   <pageSetup orientation="landscape" paperSize="9"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -920,284 +1001,217 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="11.5703125" customWidth="1" min="1" max="1"/>
-    <col width="7.5703125" customWidth="1" min="2" max="2"/>
-    <col width="1.140625" customWidth="1" min="3" max="3"/>
-    <col width="11.5703125" customWidth="1" min="4" max="4"/>
-    <col width="7.5703125" customWidth="1" min="5" max="5"/>
-    <col width="1.28515625" customWidth="1" min="6" max="6"/>
-    <col width="11.5703125" customWidth="1" min="7" max="7"/>
-    <col width="7.5703125" customWidth="1" min="8" max="8"/>
-    <col width="6.42578125" customWidth="1" min="9" max="9"/>
-    <col width="1.140625" customWidth="1" min="10" max="10"/>
-    <col width="4.42578125" customWidth="1" min="11" max="11"/>
-    <col width="12.7109375" customWidth="1" min="12" max="12"/>
+    <col width="11.5703125" customWidth="1" style="7" min="1" max="1"/>
+    <col width="7.5703125" customWidth="1" style="7" min="2" max="2"/>
+    <col width="1.140625" customWidth="1" style="7" min="3" max="3"/>
+    <col width="11.5703125" customWidth="1" style="7" min="4" max="4"/>
+    <col width="7.5703125" customWidth="1" style="7" min="5" max="5"/>
+    <col width="1.28515625" customWidth="1" style="7" min="6" max="6"/>
+    <col width="11.5703125" customWidth="1" style="7" min="7" max="7"/>
+    <col width="7.5703125" customWidth="1" style="7" min="8" max="8"/>
+    <col width="6.42578125" customWidth="1" style="7" min="9" max="9"/>
+    <col width="1.140625" customWidth="1" style="7" min="10" max="10"/>
+    <col width="4.42578125" customWidth="1" style="7" min="11" max="11"/>
+    <col width="12.7109375" customWidth="1" style="7" min="12" max="12"/>
+    <col width="9.140625" customWidth="1" style="7" min="13" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.1" customHeight="1">
+    <row r="1" ht="14.1" customHeight="1" s="7">
       <c r="A1" s="1" t="n"/>
-      <c r="E1" s="2">
-        <f>ID!M19</f>
-        <v/>
-      </c>
-      <c r="F1" s="3" t="n"/>
-      <c r="G1" s="3" t="n"/>
-      <c r="H1" s="3" t="n"/>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>*000000000000*</t>
+        </is>
+      </c>
       <c r="I1" s="4">
         <f>G4</f>
         <v/>
       </c>
       <c r="J1" s="5" t="n"/>
-      <c r="K1" s="6">
-        <f>ID!M19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="2" ht="14.1" customHeight="1">
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-    </row>
-    <row r="3" ht="5.85" customHeight="1">
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>*000000000000*</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14.1" customHeight="1" s="7"/>
+    <row r="3" ht="5.85" customHeight="1" s="7">
       <c r="E3" s="1" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-    </row>
-    <row r="4" ht="15.6" customHeight="1">
-      <c r="E4" s="7" t="inlineStr">
+    </row>
+    <row r="4" ht="15.6" customHeight="1" s="7">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>AU/Pos</t>
         </is>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="9">
         <f>'Glas-Etikette'!G4</f>
         <v/>
       </c>
-      <c r="H4" s="8">
+      <c r="H4" s="9">
         <f>'Glas-Etikette'!H4</f>
         <v/>
       </c>
-      <c r="I4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
-    </row>
-    <row r="5" ht="15" customHeight="1">
-      <c r="E5" s="7" t="inlineStr">
+    </row>
+    <row r="5" ht="15" customHeight="1" s="7">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Délai</t>
         </is>
       </c>
-      <c r="G5" s="27">
+      <c r="G5" s="10">
         <f>'Glas-Etikette'!G5</f>
         <v/>
       </c>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="K5" s="3" t="n"/>
-    </row>
-    <row r="6" ht="15" customHeight="1">
+    </row>
+    <row r="6" ht="15" customHeight="1" s="7">
       <c r="A6" s="1" t="n"/>
-      <c r="E6" s="7" t="n"/>
-      <c r="G6" s="24" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="K6" s="3" t="n"/>
-    </row>
-    <row r="7" ht="11.85" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="E6" s="8" t="n"/>
+      <c r="G6" s="25" t="n"/>
+    </row>
+    <row r="7" ht="11.85" customHeight="1" s="7">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="I7" s="3" t="n"/>
-      <c r="K7" s="3" t="n"/>
-    </row>
-    <row r="8" ht="15.6" customHeight="1">
-      <c r="A8" s="10">
+    </row>
+    <row r="8" ht="15.6" customHeight="1" s="7">
+      <c r="A8" s="11">
         <f>'Glas-Etikette'!A8</f>
         <v/>
       </c>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
-      <c r="I8" s="11" t="n"/>
-      <c r="K8" s="3" t="n"/>
-    </row>
-    <row r="9" ht="5.85" customHeight="1">
-      <c r="A9" s="7" t="n"/>
-      <c r="I9" s="28">
+      <c r="I8" s="12" t="n"/>
+    </row>
+    <row r="9" ht="5.85" customHeight="1" s="7">
+      <c r="A9" s="8" t="n"/>
+      <c r="I9" s="13">
         <f>H4</f>
         <v/>
       </c>
-      <c r="K9" s="3" t="n"/>
-    </row>
-    <row r="10" ht="14.1" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
+    </row>
+    <row r="10" ht="14.1" customHeight="1" s="7">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Commission</t>
         </is>
       </c>
-      <c r="I10" s="3" t="n"/>
-      <c r="K10" s="3" t="n"/>
-    </row>
-    <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="10">
+    </row>
+    <row r="11" ht="15" customHeight="1" s="7">
+      <c r="A11" s="11">
         <f>'Glas-Etikette'!A11</f>
         <v/>
       </c>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
-      <c r="I11" s="3" t="n"/>
-      <c r="K11" s="3" t="n"/>
-    </row>
-    <row r="12" ht="5.85" customHeight="1">
-      <c r="A12" s="7" t="n"/>
-      <c r="I12" s="3" t="n"/>
-      <c r="K12" s="3" t="n"/>
-    </row>
-    <row r="13" ht="14.1" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
+    </row>
+    <row r="12" ht="5.85" customHeight="1" s="7">
+      <c r="A12" s="8" t="n"/>
+    </row>
+    <row r="13" ht="14.1" customHeight="1" s="7">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Pos. de client</t>
         </is>
       </c>
-      <c r="I13" s="3" t="n"/>
-      <c r="K13" s="3" t="n"/>
-    </row>
-    <row r="14" ht="15" customHeight="1">
-      <c r="A14" s="10">
+    </row>
+    <row r="14" ht="15" customHeight="1" s="7">
+      <c r="A14" s="11">
         <f>IF('Glas-Etikette'!A14="","",'Glas-Etikette'!A14)</f>
         <v/>
       </c>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
-      <c r="K14" s="3" t="n"/>
-    </row>
-    <row r="15" ht="13.5" customHeight="1">
-      <c r="A15" s="13" t="n"/>
-      <c r="I15" s="3" t="n"/>
-      <c r="K15" s="14">
+    </row>
+    <row r="15" ht="13.5" customHeight="1" s="7">
+      <c r="A15" s="14" t="n"/>
+      <c r="K15" s="15">
         <f>'Glas-Etikette'!K15</f>
         <v/>
       </c>
     </row>
-    <row r="16" ht="14.1" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
+    <row r="16" ht="14.1" customHeight="1" s="7">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Verre feuilleté et verre de sécurité feuilleté avec exigence de résistance au feu</t>
         </is>
       </c>
-      <c r="K16" s="3" t="n"/>
-    </row>
-    <row r="17" ht="15.6" customHeight="1">
-      <c r="A17" s="10">
+    </row>
+    <row r="17" ht="15.6" customHeight="1" s="7">
+      <c r="A17" s="11">
         <f>'Glas-Etikette'!A17</f>
         <v/>
       </c>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n"/>
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="n"/>
-      <c r="F17" s="3" t="n"/>
-      <c r="G17" s="3" t="n"/>
-      <c r="H17" s="3" t="n"/>
-      <c r="I17" s="3" t="n"/>
-      <c r="K17" s="3" t="n"/>
-    </row>
-    <row r="18" ht="5.85" customHeight="1">
-      <c r="A18" s="7" t="n"/>
-      <c r="K18" s="3" t="n"/>
-    </row>
-    <row r="19" ht="15.6" customHeight="1">
-      <c r="A19" s="16" t="inlineStr">
+    </row>
+    <row r="18" ht="5.85" customHeight="1" s="7">
+      <c r="A18" s="8" t="n"/>
+    </row>
+    <row r="19" ht="15.6" customHeight="1" s="7">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>Quantité [Pcs]</t>
         </is>
       </c>
-      <c r="B19" s="17">
+      <c r="B19" s="18">
         <f>'Glas-Etikette'!B19</f>
         <v/>
       </c>
-      <c r="D19" s="16" t="inlineStr">
+      <c r="D19" s="17" t="inlineStr">
         <is>
           <t>Largeur [mm]</t>
         </is>
       </c>
-      <c r="E19" s="18">
+      <c r="E19" s="19">
         <f>'Glas-Etikette'!E19</f>
         <v/>
       </c>
-      <c r="G19" s="16" t="inlineStr">
+      <c r="G19" s="17" t="inlineStr">
         <is>
           <t>Hauteur [mm]</t>
         </is>
       </c>
-      <c r="H19" s="18">
+      <c r="H19" s="19">
         <f>'Glas-Etikette'!H19</f>
         <v/>
       </c>
-      <c r="K19" s="3" t="n"/>
-    </row>
-    <row r="20" ht="15.6" customHeight="1">
-      <c r="A20" s="16" t="inlineStr">
+    </row>
+    <row r="20" ht="15.6" customHeight="1" s="7">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Surface [m²]</t>
         </is>
       </c>
-      <c r="B20" s="19">
+      <c r="B20" s="20">
         <f>'Glas-Etikette'!B20</f>
         <v/>
       </c>
-      <c r="D20" s="16" t="inlineStr">
+      <c r="D20" s="17" t="inlineStr">
         <is>
           <t>Circonfér. [ml]</t>
         </is>
       </c>
-      <c r="E20" s="19">
+      <c r="E20" s="20">
         <f>'Glas-Etikette'!E20</f>
         <v/>
       </c>
-      <c r="G20" s="16" t="inlineStr">
+      <c r="G20" s="17" t="inlineStr">
         <is>
           <t>Poids [kg]</t>
         </is>
       </c>
-      <c r="H20" s="29">
+      <c r="H20" s="21">
         <f>'Glas-Etikette'!H20</f>
         <v/>
       </c>
-      <c r="K20" s="3" t="n"/>
-    </row>
-    <row r="21" ht="13.5" customHeight="1">
+    </row>
+    <row r="21" ht="13.5" customHeight="1" s="7">
       <c r="A21" s="1" t="n"/>
-      <c r="K21" s="3" t="n"/>
-    </row>
-    <row r="22" ht="11.85" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
+    </row>
+    <row r="22" ht="11.85" customHeight="1" s="7">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Enlever l'etiquette immédiatement après la pose.</t>
         </is>
       </c>
-      <c r="G22" s="21" t="n">
+      <c r="G22" s="22" t="n">
         <v>24</v>
       </c>
       <c r="H22" s="1" t="inlineStr">
@@ -1205,20 +1219,18 @@
           <t>EN 14449</t>
         </is>
       </c>
-      <c r="K22" s="3" t="n"/>
-    </row>
-    <row r="23" ht="11.85" customHeight="1">
-      <c r="A23" s="22" t="inlineStr">
+    </row>
+    <row r="23" ht="11.85" customHeight="1" s="7">
+      <c r="A23" s="23" t="inlineStr">
         <is>
           <t>CDR Glas AG | 3253 Schnottwil | 032 312 03 00 | www.cdr.ch</t>
         </is>
       </c>
-      <c r="G23" s="30" t="n">
+      <c r="G23" s="24" t="n">
         <v>757</v>
       </c>
-      <c r="K23" s="3" t="n"/>
-    </row>
-    <row r="27" ht="14.1" customHeight="1"/>
+    </row>
+    <row r="27" ht="14.1" customHeight="1" s="7"/>
   </sheetData>
   <mergeCells count="30">
     <mergeCell ref="A9:H9"/>
@@ -1245,8 +1257,8 @@
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="K1:K14"/>
+    <mergeCell ref="A8:H8"/>
     <mergeCell ref="K15:K23"/>
-    <mergeCell ref="A8:H8"/>
     <mergeCell ref="A1:D5"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A13:H13"/>
@@ -1254,5 +1266,6 @@
   </mergeCells>
   <pageMargins left="0.07874015748031496" right="0.07874015748031496" top="0.07874015748031496" bottom="0" header="0" footer="0"/>
   <pageSetup orientation="landscape" paperSize="9"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>